<commit_message>
Fix CAN tooltip positioning in maximized and fullscreen modes - Use Wayland-compatible positioning relative to the app window. - Keep Watch List and message-table popups within visible boundaries. - Reposition changing tooltips correctly while they’re open. - Preserve complete CAN details and History text. - Add regression checks for windowed, maximized and fullscreen modes. Validation: clean build; Wayland placement checks passed for both views at left, middle and right positions. User confirmed the fix works.
</commit_message>
<xml_diff>
--- a/CAN Bus Scheme 23-09-26.xlsx
+++ b/CAN Bus Scheme 23-09-26.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andy donegan\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B3ACE1B9-28E6-4935-B89D-98CC87DCB95D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E87867A-0D5D-4D20-97EB-2E0ACA4DDCF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="2" r:id="rId1"/>
@@ -6268,7 +6268,7 @@
         <v>173</v>
       </c>
       <c r="F171" s="16" t="s">
-        <v>337</v>
+        <v>315</v>
       </c>
       <c r="G171" s="17"/>
     </row>

</xml_diff>